<commit_message>
Add sample rows to expense workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016F28mx3pdxH3gHrr1AEoWb
</commit_message>
<xml_diff>
--- a/expense-agent-hooks/expense_policy.xlsx
+++ b/expense-agent-hooks/expense_policy.xlsx
@@ -155,8 +155,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="AuditLog" displayName="AuditLog" ref="A1:G2" headerRowCount="1">
-  <autoFilter ref="A1:G2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="AuditLog" displayName="AuditLog" ref="A1:G6" headerRowCount="1">
+  <autoFilter ref="A1:G6"/>
   <tableColumns count="7">
     <tableColumn id="1" name="timestamp"/>
     <tableColumn id="2" name="user"/>
@@ -171,8 +171,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Expenses" displayName="Expenses" ref="A1:G2" headerRowCount="1">
-  <autoFilter ref="A1:G2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Expenses" displayName="Expenses" ref="A1:G4" headerRowCount="1">
+  <autoFilter ref="A1:G4"/>
   <tableColumns count="7">
     <tableColumn id="1" name="expense_id"/>
     <tableColumn id="2" name="timestamp"/>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -693,21 +693,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-14T00:00:00Z</t>
+          <t>2026-10-12T09:14:00Z</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>init</t>
+          <t>amelie.dupont@contoso.com</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Repas</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -716,12 +716,152 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>log</t>
+          <t>allow</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Ligne d'initialisation (a supprimer apres le premier vrai test)</t>
+          <t>Conforme</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-12T10:02:00Z</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>jonas.weber@contoso.com</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Repas</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>85</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>deny</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Plafond depasse : 40 EUR maximum pour Repas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-13T08:40:00Z</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>sofia.rossi@contoso.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Alcool</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>60</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>deny</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>La categorie Alcool n'est jamais remboursee.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-13T15:21:00Z</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>tom.baker@contoso.com</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Materiel</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>700</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>deny</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Plafond depasse : 500 EUR maximum pour Materiel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-14T11:05:00Z</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>tom.baker@contoso.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Materiel</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>120</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>allow</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Conforme</t>
         </is>
       </c>
     </row>
@@ -739,7 +879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -791,35 +931,105 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NDF-0000</t>
+          <t>NDF-1041</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-14T00:00:00Z</t>
+          <t>2026-10-12T09:14:00Z</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>init</t>
+          <t>amelie.dupont@contoso.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Repas</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Ligne d'initialisation (a supprimer)</t>
+          <t>Resto client Acme</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Init</t>
+          <t>Soumise</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NDF-1042</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-10-13T12:30:00Z</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>jonas.weber@contoso.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Taxi</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>45</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Gare vers site client</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Soumise</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NDF-1043</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-10-14T11:05:00Z</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>tom.baker@contoso.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Materiel</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>120</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Souris et clavier</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Soumise</t>
         </is>
       </c>
     </row>

</xml_diff>